<commit_message>
update at kis office
</commit_message>
<xml_diff>
--- a/GUI/확신도_자동생성_80_85_90도_규칙.xlsx
+++ b/GUI/확신도_자동생성_80_85_90도_규칙.xlsx
@@ -553,7 +553,7 @@
         <v>0.4416881357732863</v>
       </c>
       <c r="G3" t="n">
-        <v>0.1482917252182026</v>
+        <v>0.1482917314217094</v>
       </c>
       <c r="H3" t="n">
         <v>75164</v>
@@ -588,7 +588,7 @@
         <v>0</v>
       </c>
       <c r="G4" t="n">
-        <v>0.02893559331075378</v>
+        <v>0.0289355933104418</v>
       </c>
       <c r="H4" t="n">
         <v>101141</v>
@@ -1440,16 +1440,16 @@
         <v>85</v>
       </c>
       <c r="B3" t="n">
-        <v>0.9999999963395849</v>
+        <v>0.9999997524738394</v>
       </c>
       <c r="C3" t="n">
-        <v>3.660415148588893e-09</v>
+        <v>2.475259698534553e-07</v>
       </c>
       <c r="D3" t="n">
-        <v>0</v>
+        <v>1.892315479089172e-13</v>
       </c>
       <c r="E3" t="n">
-        <v>0</v>
+        <v>1.486537805552592e-15</v>
       </c>
       <c r="F3" t="n">
         <v>0.3</v>
@@ -1460,16 +1460,16 @@
         <v>90</v>
       </c>
       <c r="B4" t="n">
-        <v>0.8802696457134092</v>
+        <v>0.8802693626121341</v>
       </c>
       <c r="C4" t="n">
-        <v>0.0438629252942775</v>
+        <v>0.04386237693622972</v>
       </c>
       <c r="D4" t="n">
-        <v>0.07586742899231338</v>
+        <v>0.07586826045163624</v>
       </c>
       <c r="E4" t="n">
-        <v>1.24683249835833e-18</v>
+        <v>0</v>
       </c>
       <c r="F4" t="n">
         <v>0.3</v>

</xml_diff>